<commit_message>
Validation batch 2: flat clip folder/paths (no dialect subfolders); regenerate matching xlsx+csv
</commit_message>
<xml_diff>
--- a/evaluation/results/validation_sample_batch2.xlsx
+++ b/evaluation/results/validation_sample_batch2.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Chittagong/Td9AAsG18Yc_0101.wav</t>
+          <t>validation_clips_batch2/Td9AAsG18Yc_0101.wav</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Barishal/4wUXS_W-mtE_0017.wav</t>
+          <t>validation_clips_batch2/4wUXS_W-mtE_0017.wav</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Narail/fjmLbMyUpG4_0280.wav</t>
+          <t>validation_clips_batch2/fjmLbMyUpG4_0280.wav</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Habiganj/zeQvYArKkoA_0016.wav</t>
+          <t>validation_clips_batch2/zeQvYArKkoA_0016.wav</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Comilla/jSAPYSksUrE_0040.wav</t>
+          <t>validation_clips_batch2/jSAPYSksUrE_0040.wav</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Sylhet/Sylhet_UK_CS__7cQH3yF9JmY_0008.wav</t>
+          <t>validation_clips_batch2/Sylhet_UK_CS__7cQH3yF9JmY_0008.wav</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Khulna/sm4X-UZrDuk_0011.wav</t>
+          <t>validation_clips_batch2/sm4X-UZrDuk_0011.wav</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Mymensingh/lmFwOoYlvks_0008.wav</t>
+          <t>validation_clips_batch2/lmFwOoYlvks_0008.wav</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Narail/maQUmuSY4tE_0018.wav</t>
+          <t>validation_clips_batch2/maQUmuSY4tE_0018.wav</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Old_Dhaka/VDa4ROkXAH8_0021.wav</t>
+          <t>validation_clips_batch2/VDa4ROkXAH8_0021.wav</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Noakhali/zNkcdb7zV8E_0015.wav</t>
+          <t>validation_clips_batch2/zNkcdb7zV8E_0015.wav</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Barishal/RXp9ycL_7Sg_0139.wav</t>
+          <t>validation_clips_batch2/RXp9ycL_7Sg_0139.wav</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Tangail/XpuOITjXlWc_0030.wav</t>
+          <t>validation_clips_batch2/XpuOITjXlWc_0030.wav</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Rangpur/9B4MlWB6_F0_0051.wav</t>
+          <t>validation_clips_batch2/9B4MlWB6_F0_0051.wav</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Rangpur/rOdVwC5GXic_0011.wav</t>
+          <t>validation_clips_batch2/rOdVwC5GXic_0011.wav</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Khulna/ej9sBQ3WKGo_0045.wav</t>
+          <t>validation_clips_batch2/ej9sBQ3WKGo_0045.wav</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Habiganj/YfPvPjHvq10_0003.wav</t>
+          <t>validation_clips_batch2/YfPvPjHvq10_0003.wav</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Kishoreganj/WZTks_8AtCs_0335.wav</t>
+          <t>validation_clips_batch2/WZTks_8AtCs_0335.wav</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Comilla/PsAaNUM0U7g_0038.wav</t>
+          <t>validation_clips_batch2/PsAaNUM0U7g_0038.wav</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Old_Dhaka/z9CMHyV8FUo_0020.wav</t>
+          <t>validation_clips_batch2/z9CMHyV8FUo_0020.wav</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Noakhali/zNkcdb7zV8E_0014.wav</t>
+          <t>validation_clips_batch2/zNkcdb7zV8E_0014.wav</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Narsingdi/82zDNyZziuY_0007.wav</t>
+          <t>validation_clips_batch2/82zDNyZziuY_0007.wav</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Tangail/yz2ZrueAmTo_0002.wav</t>
+          <t>validation_clips_batch2/yz2ZrueAmTo_0002.wav</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Mymensingh/lmFwOoYlvks_0018.wav</t>
+          <t>validation_clips_batch2/lmFwOoYlvks_0018.wav</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Sandwip/ufQHtELQPxc_0016.wav</t>
+          <t>validation_clips_batch2/ufQHtELQPxc_0016.wav</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Kishoreganj/WZTks_8AtCs_0402.wav</t>
+          <t>validation_clips_batch2/WZTks_8AtCs_0402.wav</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Chittagong/Td9AAsG18Yc_0068.wav</t>
+          <t>validation_clips_batch2/Td9AAsG18Yc_0068.wav</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Sylhet/444kGnbriMM_0033.wav</t>
+          <t>validation_clips_batch2/444kGnbriMM_0033.wav</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Sandwip/4kWyFSQhJpc_0012.wav</t>
+          <t>validation_clips_batch2/4kWyFSQhJpc_0012.wav</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>validation_clips_batch2/Narsingdi/TJwg_JeonRo_0014.wav</t>
+          <t>validation_clips_batch2/TJwg_JeonRo_0014.wav</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">

</xml_diff>